<commit_message>
estado a reunión con Laura
</commit_message>
<xml_diff>
--- a/originales/respuestas/2025/01. Calificadas/bucle p1/Agencia Analítica De Datos.xlsx
+++ b/originales/respuestas/2025/01. Calificadas/bucle p1/Agencia Analítica De Datos.xlsx
@@ -1537,15 +1537,25 @@
         <v>22</v>
       </c>
       <c r="G2" s="5"/>
-      <c r="H2" s="7"/>
+      <c r="H2" s="7">
+        <v>5.0</v>
+      </c>
       <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
+      <c r="J2" s="7">
+        <v>5.0</v>
+      </c>
       <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
+      <c r="L2" s="7">
+        <v>5.0</v>
+      </c>
       <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
+      <c r="N2" s="7">
+        <v>5.0</v>
+      </c>
       <c r="O2" s="5"/>
-      <c r="P2" s="5"/>
+      <c r="P2" s="7">
+        <v>4.0</v>
+      </c>
       <c r="Q2" s="5"/>
       <c r="R2" s="8"/>
       <c r="S2" s="8"/>

</xml_diff>